<commit_message>
feat: align Excel import with manual project form
Precondition (per-test-case):
- Moved from header metadata to a 'Precondition' column in the test
  case section of the Excel template
- Import parser now reads precondition from each test case row and
  writes it to test_cases.precondition during transactional import
- Manual TC form already had precondition — no change needed there

Scope & Criteria (project-level):
- Added header rows for Objectives, In Scope, Out of Scope, Entry
  Criteria, Exit Criteria to the Excel template
- Import parser reads these from header metadata
- Frontend import wizard preview shows editable scope/criteria fields
  and sends them when creating the project (POST /api/projects)
- Entry Criteria falls back to the old precondition header for
  backward compatibility

Demo fixture updated with new columns and header rows.
</commit_message>
<xml_diff>
--- a/artifacts/api-server/src/__tests__/fixtures/valid-test-plan.xlsx
+++ b/artifacts/api-server/src/__tests__/fixtures/valid-test-plan.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -441,193 +441,180 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Pre-condition :</v>
+        <v>Objectives:</v>
       </c>
       <c r="B6" t="str">
-        <v>User is logged in</v>
+        <v>Verify the core banking workflows for the Q4 release.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>In Scope:</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Mobile transfer, account linking, biometric login</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Use Case UC-01: Verify Login</v>
+        <v>Out of Scope:</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Web banking, ATM flow, fraud detection</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Test Case#</v>
+        <v>Entry Criteria:</v>
       </c>
       <c r="B9" t="str">
-        <v>Test Title</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Test Steps</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Test Data</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Expected Result</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Actual Result</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Status(Pass/Fail)</v>
-      </c>
-      <c r="H9" t="str">
-        <v>Notes</v>
+        <v>Build deployed to staging, test accounts provisioned</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>1</v>
+        <v>Exit Criteria:</v>
       </c>
       <c r="B10" t="str">
-        <v>Valid login</v>
-      </c>
-      <c r="C10" t="str">
-        <v>(i) Enter username</v>
-      </c>
-      <c r="D10" t="str">
-        <v>admin</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Login succeeds</v>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v>(ii) Enter password</v>
-      </c>
-      <c r="D11" t="str">
-        <v>pass123</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Password accepted</v>
-      </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v/>
+        <v>100% critical scenarios passed, no P1 defects open</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <v>(iii) Click login</v>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v>Dashboard visible</v>
-      </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
-      <c r="H12" t="str">
-        <v/>
+        <v>Use Case UC-01: Verify Login</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>2</v>
+        <v>Test Case#</v>
       </c>
       <c r="B13" t="str">
-        <v>Invalid login</v>
+        <v>Test Title</v>
       </c>
       <c r="C13" t="str">
-        <v>Enter wrong credentials</v>
+        <v>Test Steps</v>
       </c>
       <c r="D13" t="str">
-        <v>bad/pass</v>
+        <v>Test Data</v>
       </c>
       <c r="E13" t="str">
-        <v>Error shown</v>
+        <v>Expected Result</v>
       </c>
       <c r="F13" t="str">
-        <v/>
+        <v>Actual Result</v>
       </c>
       <c r="G13" t="str">
-        <v/>
+        <v>Status(Pass/Fail)</v>
       </c>
       <c r="H13" t="str">
-        <v/>
+        <v>Notes</v>
+      </c>
+      <c r="I13" t="str">
+        <v>Precondition</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>1</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Valid login</v>
+      </c>
+      <c r="C14" t="str">
+        <v>(i) Enter username</v>
+      </c>
+      <c r="D14" t="str">
+        <v>admin</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Login succeeds</v>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+      <c r="I14" t="str">
+        <v>User must be registered</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Use Case UC-02: Invoice Management</v>
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v>(ii) Enter password</v>
+      </c>
+      <c r="D15" t="str">
+        <v>pass123</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Password accepted</v>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+      <c r="I15" t="str">
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Test Case#</v>
+        <v/>
       </c>
       <c r="B16" t="str">
-        <v>Test Title</v>
+        <v/>
       </c>
       <c r="C16" t="str">
-        <v>Test Steps</v>
+        <v>(iii) Click login</v>
       </c>
       <c r="D16" t="str">
-        <v>Test Data</v>
+        <v/>
       </c>
       <c r="E16" t="str">
-        <v>Expected Result</v>
+        <v>Dashboard visible</v>
       </c>
       <c r="F16" t="str">
-        <v>Actual Result</v>
+        <v/>
       </c>
       <c r="G16" t="str">
-        <v>Status(Pass/Fail)</v>
+        <v/>
       </c>
       <c r="H16" t="str">
-        <v>Notes</v>
+        <v/>
+      </c>
+      <c r="I16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B17" t="str">
-        <v>Create invoice</v>
+        <v>Invalid login</v>
       </c>
       <c r="C17" t="str">
-        <v>Fill invoice form</v>
+        <v>Enter wrong credentials</v>
       </c>
       <c r="D17" t="str">
-        <v>inv-001</v>
+        <v>bad/pass</v>
       </c>
       <c r="E17" t="str">
-        <v>Invoice created</v>
+        <v>Error shown</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -638,67 +625,139 @@
       <c r="H17" t="str">
         <v/>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>1A</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Approve invoice</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Click approve</v>
-      </c>
-      <c r="D18" t="str">
-        <v>inv-001</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Status changes to approved</v>
-      </c>
-      <c r="F18" t="str">
-        <v/>
-      </c>
-      <c r="G18" t="str">
-        <v/>
-      </c>
-      <c r="H18" t="str">
-        <v/>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Use Case UC-02: Invoice Management</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Use Case UC-03: Empty use case</v>
+        <v>Test Case#</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Test Title</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Test Steps</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Test Data</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Expected Result</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Actual Result</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Status(Pass/Fail)</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="I20" t="str">
+        <v>Precondition</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>1</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Create invoice</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Fill invoice form</v>
+      </c>
+      <c r="D21" t="str">
+        <v>inv-001</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Invoice created</v>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v>User logged in with billing role</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>1A</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Approve invoice</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Click approve</v>
+      </c>
+      <c r="D22" t="str">
+        <v>inv-001</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Status changes to approved</v>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Use Case UC-03: Empty use case</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
         <v>Test Case#</v>
       </c>
-      <c r="B21" t="str">
+      <c r="B25" t="str">
         <v>Test Title</v>
       </c>
-      <c r="C21" t="str">
+      <c r="C25" t="str">
         <v>Test Steps</v>
       </c>
-      <c r="D21" t="str">
+      <c r="D25" t="str">
         <v>Test Data</v>
       </c>
-      <c r="E21" t="str">
+      <c r="E25" t="str">
         <v>Expected Result</v>
       </c>
-      <c r="F21" t="str">
+      <c r="F25" t="str">
         <v>Actual Result</v>
       </c>
-      <c r="G21" t="str">
+      <c r="G25" t="str">
         <v>Status(Pass/Fail)</v>
       </c>
-      <c r="H21" t="str">
+      <c r="H25" t="str">
         <v>Notes</v>
+      </c>
+      <c r="I25" t="str">
+        <v>Precondition</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I25"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>